<commit_message>
Add USDA abridged fallback, USDA nutrient names, cooking_method, and data templates
- Add abridged format fallback in fetch_food_data() for FDC IDs that return 404
  with full format (e.g., Foundation entry 748967)
- Add NUTRIENT_NUMBER_TO_ID mapping for abridged-to-standard nutrient ID translation
- Add usda_name field to all 50 FEDIAF nutrients in fediaf_nutrients.py
- Fix usda_nutrient_name being NULL for supplement and no-USDA-data flows
- Add cooking_method column to ingredients schema and user prompts
- Add data export CSVs and Excel templates for ingredient analysis

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/ingredient prices.xlsx
+++ b/data/ingredient prices.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sderhami/Documents/Apps/nutDataGen/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30EB5A47-2F00-7249-97B3-E5E73535954F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{366CE407-65E9-674F-A3CA-19419A1BFD33}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-41800" yWindow="5480" windowWidth="28040" windowHeight="17440" xr2:uid="{37331FF1-933B-3840-9A66-BE0F7B949161}"/>
+    <workbookView xWindow="-33640" yWindow="10720" windowWidth="28040" windowHeight="17440" xr2:uid="{37331FF1-933B-3840-9A66-BE0F7B949161}"/>
   </bookViews>
   <sheets>
     <sheet name="Ingredients" sheetId="1" r:id="rId1"/>
@@ -35,8 +35,118 @@
 </workbook>
 </file>
 
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>Shahab Derhami</author>
+  </authors>
+  <commentList>
+    <comment ref="B5" authorId="0" shapeId="0" xr:uid="{2015DF91-C3EF-8A49-827B-29ED0984C71D}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Shahab Derhami:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+            <scheme val="minor"/>
+          </rPr>
+          <t>1 lb (454g) of shell-on blue mussels → approximately 100–115g of raw meat. Price was $4/lb with shells</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B6" authorId="0" shapeId="0" xr:uid="{3B9D9B57-98C0-5140-924F-C3A7C058CBB3}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Shahab Derhami:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>price per egg</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="C6" authorId="0" shapeId="0" xr:uid="{008EEC43-5EE2-884B-90B2-4B44E74430AF}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Shahab Derhami:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>one large egg is 50g edible</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="24">
   <si>
     <t>Price per pound</t>
   </si>
@@ -90,6 +200,24 @@
   </si>
   <si>
     <t>chicken heart raw</t>
+  </si>
+  <si>
+    <t>KI stock solution</t>
+  </si>
+  <si>
+    <t>Blue mussel raw</t>
+  </si>
+  <si>
+    <t>chicken egg raw</t>
+  </si>
+  <si>
+    <t>Pure Encapsulations Manganese</t>
+  </si>
+  <si>
+    <t>capsule</t>
+  </si>
+  <si>
+    <t>beef liver raw</t>
   </si>
 </sst>
 </file>
@@ -100,7 +228,7 @@
     <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="165" formatCode="_(&quot;$&quot;* #,##0.0000_);_(&quot;$&quot;* \(#,##0.0000\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -111,6 +239,26 @@
     <font>
       <sz val="12"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -457,8 +605,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0E2FD49C-90A6-2545-B1AD-F87C0CE7D7C6}">
-  <dimension ref="A1:E4"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0E2FD49C-90A6-2545-B1AD-F87C0CE7D7C6}">
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="31.83203125" bestFit="1" customWidth="1"/>
@@ -528,14 +676,61 @@
         <v>4.3995494861326203E-3</v>
       </c>
     </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>19</v>
+      </c>
+      <c r="B5" s="1">
+        <v>16</v>
+      </c>
+      <c r="C5">
+        <v>454.59199999999998</v>
+      </c>
+      <c r="D5" s="3">
+        <f>B5/C5</f>
+        <v>3.5196395889060962E-2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>20</v>
+      </c>
+      <c r="B6" s="1">
+        <f>3/12</f>
+        <v>0.25</v>
+      </c>
+      <c r="C6">
+        <v>50</v>
+      </c>
+      <c r="D6" s="3">
+        <f>B6/C6</f>
+        <v>5.0000000000000001E-3</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>23</v>
+      </c>
+      <c r="B7" s="1">
+        <v>4.99</v>
+      </c>
+      <c r="C7">
+        <v>454.59199999999998</v>
+      </c>
+      <c r="D7" s="3">
+        <f>B7/C7</f>
+        <v>1.0976875967900888E-2</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <legacyDrawing r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{88BF1BC6-491C-2C49-8D01-A8FB464A2033}">
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="31.83203125" bestFit="1" customWidth="1"/>
@@ -651,6 +846,48 @@
         <v>0.64902998236331566</v>
       </c>
     </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>18</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C6">
+        <v>1</v>
+      </c>
+      <c r="D6" s="1">
+        <v>30</v>
+      </c>
+      <c r="E6">
+        <v>57</v>
+      </c>
+      <c r="F6" s="4">
+        <f>D6/E6</f>
+        <v>0.52631578947368418</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>21</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C7">
+        <v>1</v>
+      </c>
+      <c r="D7" s="1">
+        <v>13</v>
+      </c>
+      <c r="E7">
+        <v>60</v>
+      </c>
+      <c r="F7" s="1">
+        <f>D7/E7</f>
+        <v>0.21666666666666667</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
WIP: nutrient data-gen improvements (schema, backfill, USDA, tests)
Accumulated working changes on main prior to branching for the nutrient-CV
extraction work:
- Alembic migrations: source 'none' for non-supplement rows; base category
  for water/other; 'boiled_drained' cooking method; catch-up ingredient
  source URLs.
- backfill_nutrients.py: SR Legacy + Foundation nutrient backfill with AI
  value selection.
- Updates to database.py, main.py, usda_api.py, user_interaction.py,
  fediaf_nutrients.py, config.py, supplement_template.py + tests + data
  templates.
- gitignore DB dumps under backups/.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/ingredient prices.xlsx
+++ b/data/ingredient prices.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sderhami/Documents/Apps/nutDataGen/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{366CE407-65E9-674F-A3CA-19419A1BFD33}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7FAD762-7815-7548-8036-1C1E8D81B0BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-33640" yWindow="10720" windowWidth="28040" windowHeight="17440" xr2:uid="{37331FF1-933B-3840-9A66-BE0F7B949161}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17180" activeTab="1" xr2:uid="{37331FF1-933B-3840-9A66-BE0F7B949161}"/>
   </bookViews>
   <sheets>
     <sheet name="Ingredients" sheetId="1" r:id="rId1"/>
@@ -141,12 +141,263 @@
         </r>
       </text>
     </comment>
+    <comment ref="B11" authorId="0" shapeId="0" xr:uid="{8BEAE438-2264-1D41-B7BA-BE995EB5B65C}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Shahab Derhami:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>price per egg</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="C11" authorId="0" shapeId="0" xr:uid="{47A5D6D0-FD84-A249-8F1A-1C6D17F3C3E9}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Shahab Derhami:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>one large egg is 50g out of which 33g is white</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="A13" authorId="0" shapeId="0" xr:uid="{C9FB0C0D-FCB7-5245-AD61-94CE0D60BE04}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Shahab Derhami:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>originally, enterd in the db using 100g chicken bones. then added 25% water to it, portionqty updated to 125 and moisture increased from 46.2g to 71.2g</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B13" authorId="0" shapeId="0" xr:uid="{32AE55D4-FAF6-4949-B2DE-23DC5F41AF81}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Shahab Derhami:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Estimated price of chicken bones</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B19" authorId="0" shapeId="0" xr:uid="{749EFB35-6A40-4E42-832C-D5BCAD2B7001}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Shahab Derhami:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>price per egg</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="C19" authorId="0" shapeId="0" xr:uid="{25189C65-6FFC-4243-BE74-DA9BFE05C3DF}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Shahab Derhami:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>one large egg is 50g out of which 33g is white and 17g is yolk</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>Shahab Derhami</author>
+  </authors>
+  <commentList>
+    <comment ref="A13" authorId="0" shapeId="0" xr:uid="{D0E1B177-7AC9-D746-A8B7-A052B12E139B}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Shahab Derhami:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">had to mix the product label with ai validaton. ran ai validation once, then updated the values with product label and another round of ai validation by claude opus 4.7
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>2nd edit: had to convert the base unit to tbsp because of the product label mismatch. Originally entered for 100g portion. Portion QTY=100g/8, ME/unit=3.75*8</t>
+        </r>
+      </text>
+    </comment>
   </commentList>
 </comments>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="58">
   <si>
     <t>Price per pound</t>
   </si>
@@ -218,6 +469,108 @@
   </si>
   <si>
     <t>beef liver raw</t>
+  </si>
+  <si>
+    <t>Salmon Atlantic farm raised raw</t>
+  </si>
+  <si>
+    <t>NOW nztural vitamin E liquid</t>
+  </si>
+  <si>
+    <t>drop</t>
+  </si>
+  <si>
+    <t>chicken breast with skin raw</t>
+  </si>
+  <si>
+    <t>tilapia farm raised raw</t>
+  </si>
+  <si>
+    <t>chicken egg white raw</t>
+  </si>
+  <si>
+    <t>butternut squash raw</t>
+  </si>
+  <si>
+    <t>chicken bone meal</t>
+  </si>
+  <si>
+    <t>beef top round raw</t>
+  </si>
+  <si>
+    <t>NOW Iron 18ml</t>
+  </si>
+  <si>
+    <t>Pure copper glycinate</t>
+  </si>
+  <si>
+    <t>Zinc Gluconate Powder BulkSupplements</t>
+  </si>
+  <si>
+    <t>g</t>
+  </si>
+  <si>
+    <t>Iodized salt morton</t>
+  </si>
+  <si>
+    <t>Nutritional yeast sari</t>
+  </si>
+  <si>
+    <t>turkey thigh meat and skin raw</t>
+  </si>
+  <si>
+    <t>turkey breast meat and skin raw</t>
+  </si>
+  <si>
+    <t>turkey heart raw</t>
+  </si>
+  <si>
+    <t>turkey liver raw</t>
+  </si>
+  <si>
+    <t>chicken egg yolk raw</t>
+  </si>
+  <si>
+    <t>choline now supplements</t>
+  </si>
+  <si>
+    <t>white rice unenriched raw</t>
+  </si>
+  <si>
+    <t>Potassium Iodine MaryRuth</t>
+  </si>
+  <si>
+    <t>Beef chuck roast boneless raw</t>
+  </si>
+  <si>
+    <t>Pumpkin raw</t>
+  </si>
+  <si>
+    <t>Pork loin bonless raw</t>
+  </si>
+  <si>
+    <t>Pork shoulder boneless raw</t>
+  </si>
+  <si>
+    <t>Zinc Gluconate Powder Now</t>
+  </si>
+  <si>
+    <t>tablet</t>
+  </si>
+  <si>
+    <t>Potassium Gluconate now</t>
+  </si>
+  <si>
+    <t>Potassium Cotrate powder now</t>
+  </si>
+  <si>
+    <t>tbsp</t>
+  </si>
+  <si>
+    <t>whole</t>
+  </si>
+  <si>
+    <t>empty shells</t>
   </si>
 </sst>
 </file>
@@ -226,7 +579,7 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
     <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="165" formatCode="_(&quot;$&quot;* #,##0.0000_);_(&quot;$&quot;* \(#,##0.0000\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="164" formatCode="_(&quot;$&quot;* #,##0.0000_);_(&quot;$&quot;* \(#,##0.0000\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
   <fonts count="5" x14ac:knownFonts="1">
     <font>
@@ -264,12 +617,24 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -285,12 +650,14 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Currency" xfId="1" builtinId="4"/>
@@ -606,7 +973,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0E2FD49C-90A6-2545-B1AD-F87C0CE7D7C6}">
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E24"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="31.83203125" bestFit="1" customWidth="1"/>
@@ -640,7 +1007,7 @@
         <v>453.59199999999998</v>
       </c>
       <c r="D2" s="3">
-        <f>B2/C2</f>
+        <f t="shared" ref="D2:D24" si="0">B2/C2</f>
         <v>1.1464046984955643E-2</v>
       </c>
       <c r="E2" s="2"/>
@@ -657,7 +1024,7 @@
         <v>453.59199999999998</v>
       </c>
       <c r="D3" s="3">
-        <f>B3/C3</f>
+        <f t="shared" si="0"/>
         <v>6.7020582373586842E-3</v>
       </c>
     </row>
@@ -669,11 +1036,11 @@
         <v>2</v>
       </c>
       <c r="C4">
-        <v>454.59199999999998</v>
+        <v>453.59199999999998</v>
       </c>
       <c r="D4" s="3">
-        <f>B4/C4</f>
-        <v>4.3995494861326203E-3</v>
+        <f t="shared" si="0"/>
+        <v>4.4092488403675552E-3</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.2">
@@ -684,11 +1051,11 @@
         <v>16</v>
       </c>
       <c r="C5">
-        <v>454.59199999999998</v>
+        <v>453.59199999999998</v>
       </c>
       <c r="D5" s="3">
-        <f>B5/C5</f>
-        <v>3.5196395889060962E-2</v>
+        <f t="shared" si="0"/>
+        <v>3.5273990722940442E-2</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.2">
@@ -703,7 +1070,7 @@
         <v>50</v>
       </c>
       <c r="D6" s="3">
-        <f>B6/C6</f>
+        <f t="shared" si="0"/>
         <v>5.0000000000000001E-3</v>
       </c>
     </row>
@@ -715,31 +1082,289 @@
         <v>4.99</v>
       </c>
       <c r="C7">
+        <v>453.59199999999998</v>
+      </c>
+      <c r="D7" s="3">
+        <f t="shared" si="0"/>
+        <v>1.1001075856717051E-2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>24</v>
+      </c>
+      <c r="B8" s="1">
+        <v>10.99</v>
+      </c>
+      <c r="C8">
+        <v>453.59199999999998</v>
+      </c>
+      <c r="D8" s="3">
+        <f t="shared" si="0"/>
+        <v>2.4228822377819717E-2</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>27</v>
+      </c>
+      <c r="B9" s="1">
+        <v>6.99</v>
+      </c>
+      <c r="C9">
+        <v>453.59199999999998</v>
+      </c>
+      <c r="D9" s="3">
+        <f t="shared" si="0"/>
+        <v>1.5410324697084605E-2</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>28</v>
+      </c>
+      <c r="B10" s="1">
+        <v>6.99</v>
+      </c>
+      <c r="C10">
+        <v>453.59199999999998</v>
+      </c>
+      <c r="D10" s="3">
+        <f t="shared" si="0"/>
+        <v>1.5410324697084605E-2</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>29</v>
+      </c>
+      <c r="B11" s="1">
+        <f>3/12</f>
+        <v>0.25</v>
+      </c>
+      <c r="C11">
+        <v>33</v>
+      </c>
+      <c r="D11" s="3">
+        <f t="shared" si="0"/>
+        <v>7.575757575757576E-3</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>30</v>
+      </c>
+      <c r="B12" s="1">
+        <v>2.4</v>
+      </c>
+      <c r="C12">
+        <v>453.59199999999998</v>
+      </c>
+      <c r="D12" s="3">
+        <f t="shared" si="0"/>
+        <v>5.2910986084410659E-3</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>31</v>
+      </c>
+      <c r="B13" s="1">
+        <v>2.99</v>
+      </c>
+      <c r="C13">
+        <v>453.59199999999998</v>
+      </c>
+      <c r="D13" s="3">
+        <f t="shared" si="0"/>
+        <v>6.5918270163494953E-3</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>32</v>
+      </c>
+      <c r="B14" s="1">
+        <v>10.49</v>
+      </c>
+      <c r="C14">
         <v>454.59199999999998</v>
       </c>
-      <c r="D7" s="3">
-        <f>B7/C7</f>
-        <v>1.0976875967900888E-2</v>
+      <c r="D14" s="3">
+        <f t="shared" si="0"/>
+        <v>2.3075637054765594E-2</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>39</v>
+      </c>
+      <c r="B15" s="1">
+        <v>5.99</v>
+      </c>
+      <c r="C15">
+        <v>454.59199999999998</v>
+      </c>
+      <c r="D15" s="3">
+        <f t="shared" si="0"/>
+        <v>1.3176650710967198E-2</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>40</v>
+      </c>
+      <c r="B16" s="1">
+        <v>7.29</v>
+      </c>
+      <c r="C16">
+        <v>454.59199999999998</v>
+      </c>
+      <c r="D16" s="3">
+        <f t="shared" si="0"/>
+        <v>1.60363578769534E-2</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>41</v>
+      </c>
+      <c r="B17" s="1">
+        <v>5</v>
+      </c>
+      <c r="C17">
+        <v>454.59199999999998</v>
+      </c>
+      <c r="D17" s="3">
+        <f t="shared" si="0"/>
+        <v>1.099887371533155E-2</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
+        <v>42</v>
+      </c>
+      <c r="B18" s="1">
+        <v>4</v>
+      </c>
+      <c r="C18">
+        <v>454.59199999999998</v>
+      </c>
+      <c r="D18" s="3">
+        <f t="shared" si="0"/>
+        <v>8.7990989722652405E-3</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A19" t="s">
+        <v>43</v>
+      </c>
+      <c r="B19" s="1">
+        <f>3/12</f>
+        <v>0.25</v>
+      </c>
+      <c r="C19">
+        <v>17</v>
+      </c>
+      <c r="D19" s="3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A20" t="s">
+        <v>45</v>
+      </c>
+      <c r="B20" s="1">
+        <f>24/15</f>
+        <v>1.6</v>
+      </c>
+      <c r="C20">
+        <v>454.59199999999998</v>
+      </c>
+      <c r="D20" s="3">
+        <f t="shared" si="0"/>
+        <v>3.5196395889060964E-3</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A21" t="s">
+        <v>47</v>
+      </c>
+      <c r="B21" s="1">
+        <v>9</v>
+      </c>
+      <c r="C21">
+        <v>454.59199999999998</v>
+      </c>
+      <c r="D21" s="3">
+        <f t="shared" si="0"/>
+        <v>1.9797972687596792E-2</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A22" t="s">
+        <v>48</v>
+      </c>
+      <c r="B22" s="1">
+        <v>3</v>
+      </c>
+      <c r="C22">
+        <v>454.59199999999998</v>
+      </c>
+      <c r="D22" s="3">
+        <f t="shared" si="0"/>
+        <v>6.59932422919893E-3</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A23" t="s">
+        <v>49</v>
+      </c>
+      <c r="B23" s="1">
+        <v>3</v>
+      </c>
+      <c r="C23">
+        <v>454.59199999999998</v>
+      </c>
+      <c r="D23" s="3">
+        <f t="shared" si="0"/>
+        <v>6.59932422919893E-3</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A24" t="s">
+        <v>50</v>
+      </c>
+      <c r="B24" s="1">
+        <v>5</v>
+      </c>
+      <c r="C24">
+        <v>454.59199999999998</v>
+      </c>
+      <c r="D24" s="3">
+        <f t="shared" si="0"/>
+        <v>1.099887371533155E-2</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
   <legacyDrawing r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{88BF1BC6-491C-2C49-8D01-A8FB464A2033}">
-  <dimension ref="A1:F7"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{88BF1BC6-491C-2C49-8D01-A8FB464A2033}">
+  <dimension ref="A1:I19"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="31.83203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="35.33203125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="22.1640625" style="1" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="32.6640625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="10.83203125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>2</v>
       </c>
@@ -758,15 +1383,21 @@
       <c r="F1" s="1" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G1" t="s">
+        <v>56</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>5</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C2">
+      <c r="C2" s="5">
         <v>0.25</v>
       </c>
       <c r="D2" s="1">
@@ -778,18 +1409,18 @@
         <v>56.75</v>
       </c>
       <c r="F2" s="4">
-        <f>D2/E2</f>
+        <f t="shared" ref="F2:F18" si="0">D2/E2</f>
         <v>0.1552422907488987</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>10</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C3">
+      <c r="C3" s="5">
         <v>0.5</v>
       </c>
       <c r="D3" s="1">
@@ -799,11 +1430,11 @@
         <v>100</v>
       </c>
       <c r="F3" s="4">
-        <f>D3/E3</f>
+        <f t="shared" si="0"/>
         <v>0.1399</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>13</v>
       </c>
@@ -820,11 +1451,11 @@
         <v>60</v>
       </c>
       <c r="F4" s="4">
-        <f>D4/E4</f>
+        <f t="shared" si="0"/>
         <v>0.25433333333333336</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>15</v>
       </c>
@@ -842,11 +1473,11 @@
         <v>28.35</v>
       </c>
       <c r="F5" s="4">
-        <f>D5/E5</f>
+        <f t="shared" si="0"/>
         <v>0.64902998236331566</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>18</v>
       </c>
@@ -863,11 +1494,11 @@
         <v>57</v>
       </c>
       <c r="F6" s="4">
-        <f>D6/E6</f>
+        <f t="shared" si="0"/>
         <v>0.52631578947368418</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>21</v>
       </c>
@@ -883,12 +1514,301 @@
       <c r="E7">
         <v>60</v>
       </c>
-      <c r="F7" s="1">
-        <f>D7/E7</f>
+      <c r="F7" s="4">
+        <f t="shared" si="0"/>
         <v>0.21666666666666667</v>
       </c>
+      <c r="G7">
+        <f>1.07/5</f>
+        <v>0.21400000000000002</v>
+      </c>
+      <c r="H7">
+        <f>0.239/5</f>
+        <v>4.7799999999999995E-2</v>
+      </c>
+      <c r="I7" s="6">
+        <f>G7-H7</f>
+        <v>0.16620000000000001</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>25</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C8">
+        <v>1</v>
+      </c>
+      <c r="D8" s="1">
+        <v>12</v>
+      </c>
+      <c r="E8">
+        <v>900</v>
+      </c>
+      <c r="F8" s="4">
+        <f t="shared" si="0"/>
+        <v>1.3333333333333334E-2</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>33</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C9">
+        <v>1</v>
+      </c>
+      <c r="D9" s="1">
+        <v>9</v>
+      </c>
+      <c r="E9">
+        <v>120</v>
+      </c>
+      <c r="F9" s="4">
+        <f t="shared" si="0"/>
+        <v>7.4999999999999997E-2</v>
+      </c>
+      <c r="G9">
+        <f>2.37/5</f>
+        <v>0.47400000000000003</v>
+      </c>
+      <c r="H9">
+        <f>0.378/5</f>
+        <v>7.5600000000000001E-2</v>
+      </c>
+      <c r="I9" s="6">
+        <f>G9-H9</f>
+        <v>0.39840000000000003</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>34</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C10">
+        <v>1</v>
+      </c>
+      <c r="D10" s="1">
+        <v>13</v>
+      </c>
+      <c r="E10">
+        <v>60</v>
+      </c>
+      <c r="F10" s="4">
+        <f t="shared" si="0"/>
+        <v>0.21666666666666667</v>
+      </c>
+      <c r="G10">
+        <f>0.989/5</f>
+        <v>0.1978</v>
+      </c>
+      <c r="H10">
+        <f>0.234/5</f>
+        <v>4.6800000000000001E-2</v>
+      </c>
+      <c r="I10" s="6">
+        <f>G10-H10</f>
+        <v>0.151</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>35</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="C11" s="5">
+        <v>0.28499999999999998</v>
+      </c>
+      <c r="D11" s="1">
+        <v>21</v>
+      </c>
+      <c r="E11">
+        <v>1754</v>
+      </c>
+      <c r="F11" s="4">
+        <f t="shared" si="0"/>
+        <v>1.1972633979475485E-2</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>37</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C12" s="5">
+        <v>0.25</v>
+      </c>
+      <c r="D12" s="1">
+        <v>3</v>
+      </c>
+      <c r="E12">
+        <v>491</v>
+      </c>
+      <c r="F12" s="4">
+        <f t="shared" si="0"/>
+        <v>6.1099796334012219E-3</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>38</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="C13">
+        <f>100/8</f>
+        <v>12.5</v>
+      </c>
+      <c r="D13" s="1">
+        <v>18</v>
+      </c>
+      <c r="E13">
+        <v>28</v>
+      </c>
+      <c r="F13" s="4">
+        <f t="shared" si="0"/>
+        <v>0.6428571428571429</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>44</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C14">
+        <v>1</v>
+      </c>
+      <c r="D14" s="1">
+        <v>10</v>
+      </c>
+      <c r="E14">
+        <v>100</v>
+      </c>
+      <c r="F14" s="4">
+        <f t="shared" si="0"/>
+        <v>0.1</v>
+      </c>
+      <c r="G14">
+        <f>4.702/5</f>
+        <v>0.94040000000000001</v>
+      </c>
+      <c r="H14">
+        <f>0.615/5</f>
+        <v>0.123</v>
+      </c>
+      <c r="I14" s="6">
+        <f>G14-H14</f>
+        <v>0.81740000000000002</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>46</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C15">
+        <v>1</v>
+      </c>
+      <c r="D15" s="1">
+        <v>16</v>
+      </c>
+      <c r="E15">
+        <v>900</v>
+      </c>
+      <c r="F15" s="4">
+        <f t="shared" si="0"/>
+        <v>1.7777777777777778E-2</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>51</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="C16">
+        <v>1</v>
+      </c>
+      <c r="D16" s="1">
+        <v>6</v>
+      </c>
+      <c r="E16">
+        <v>100</v>
+      </c>
+      <c r="F16" s="4">
+        <f t="shared" si="0"/>
+        <v>0.06</v>
+      </c>
+      <c r="G16" s="6">
+        <f>5.303/10</f>
+        <v>0.53029999999999999</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>53</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="C17">
+        <v>1</v>
+      </c>
+      <c r="D17" s="1">
+        <v>9</v>
+      </c>
+      <c r="E17">
+        <v>100</v>
+      </c>
+      <c r="F17" s="4">
+        <f t="shared" si="0"/>
+        <v>0.09</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
+        <v>54</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C18">
+        <v>0.25</v>
+      </c>
+      <c r="D18" s="1">
+        <v>12</v>
+      </c>
+      <c r="E18">
+        <v>243</v>
+      </c>
+      <c r="F18" s="4">
+        <f>D18/E18/C18</f>
+        <v>0.19753086419753085</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="B19" s="1"/>
+      <c r="F19" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <legacyDrawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update ingredient prices spreadsheet
Working-tree change to data/ingredient prices.xlsx, carried over from before
the AI-validation hardening work and committed here on request.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/ingredient prices.xlsx
+++ b/data/ingredient prices.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10125"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10726"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sderhami/Documents/Apps/nutDataGen/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7FAD762-7815-7548-8036-1C1E8D81B0BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D93D6B0-FF8F-7A44-9EC7-4A22A82D6B58}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17180" activeTab="1" xr2:uid="{37331FF1-933B-3840-9A66-BE0F7B949161}"/>
+    <workbookView xWindow="10940" yWindow="2900" windowWidth="37880" windowHeight="23820" xr2:uid="{37331FF1-933B-3840-9A66-BE0F7B949161}"/>
   </bookViews>
   <sheets>
     <sheet name="Ingredients" sheetId="1" r:id="rId1"/>
@@ -397,7 +397,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="59">
   <si>
     <t>Price per pound</t>
   </si>
@@ -571,6 +571,9 @@
   </si>
   <si>
     <t>empty shells</t>
+  </si>
+  <si>
+    <t>lamb shoulder lean only raw</t>
   </si>
 </sst>
 </file>
@@ -973,7 +976,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0E2FD49C-90A6-2545-B1AD-F87C0CE7D7C6}">
-  <dimension ref="A1:E24"/>
+  <dimension ref="A1:E25"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="31.83203125" bestFit="1" customWidth="1"/>
@@ -1007,7 +1010,7 @@
         <v>453.59199999999998</v>
       </c>
       <c r="D2" s="3">
-        <f t="shared" ref="D2:D24" si="0">B2/C2</f>
+        <f t="shared" ref="D2:D25" si="0">B2/C2</f>
         <v>1.1464046984955643E-2</v>
       </c>
       <c r="E2" s="2"/>
@@ -1344,6 +1347,21 @@
       <c r="D24" s="3">
         <f t="shared" si="0"/>
         <v>1.099887371533155E-2</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A25" t="s">
+        <v>58</v>
+      </c>
+      <c r="B25" s="1">
+        <v>15.5</v>
+      </c>
+      <c r="C25">
+        <v>454.59199999999998</v>
+      </c>
+      <c r="D25" s="3">
+        <f t="shared" si="0"/>
+        <v>3.4096508517527803E-2</v>
       </c>
     </row>
   </sheetData>
@@ -1409,7 +1427,7 @@
         <v>56.75</v>
       </c>
       <c r="F2" s="4">
-        <f t="shared" ref="F2:F18" si="0">D2/E2</f>
+        <f t="shared" ref="F2:F17" si="0">D2/E2</f>
         <v>0.1552422907488987</v>
       </c>
     </row>

</xml_diff>